<commit_message>
feat: finish project hastly
add terminal screenshot, add readme, fix typos, add my section
if anyone is reading this im so sorry
</commit_message>
<xml_diff>
--- a/Challenge4.xlsx
+++ b/Challenge4.xlsx
@@ -17,98 +17,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
-  <si>
-    <t xml:space="preserve">Item  Number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cafe item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Practice price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coffee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$2.50 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$2.00 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$3.25 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bagel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$4.00 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Breakfast Sanwhich</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$5.50 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">salad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$6.75 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Soup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$3.75 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$7.25 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pasta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$8.50 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cookie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$1.50 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muffin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$2.75 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smoothie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$4.50 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Combo Meal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$9.00 </t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -309,179 +217,118 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.33"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="0" t="s">
+      <c r="A1" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
-        <v>2</v>
+      <c r="B1" s="0" t="n">
+        <v>2.50</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>2.00</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>3.25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>4.00</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>5.50</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>6.75</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>3.75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7.25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>18</v>
+        <v>9</v>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8.50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>20</v>
+        <v>10</v>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>1.50</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>2.75</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>4.50</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>28</v>
+      <c r="B13" s="0" t="n">
+        <v>9.00</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>